<commit_message>
small fix in analysis data codebook
</commit_message>
<xml_diff>
--- a/1_data/3_AnalysisData/MetaData/codebook_AnalysisData.xlsx
+++ b/1_data/3_AnalysisData/MetaData/codebook_AnalysisData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="217">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -185,6 +185,126 @@
     <t xml:space="preserve">Animacy-Size task. Average response time on correct trials of the switch condition</t>
   </si>
   <si>
+    <t xml:space="preserve">noise_simon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">noise_flanker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">noise_globallocal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">noise_colorshape</t>
+  </si>
+  <si>
+    <t xml:space="preserve">noise_animacysize</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stai_simon_diff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stai_flanker_diff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stai_globallocal_diff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stai_colorshape_diff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stai_animacysize_diff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fl_score_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flanker task. Log-transformed Congruency effect based on mean response times (congruent - incongruent). Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fl_rt_con_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flanker task. Log-transformed Average response time on correct trials of the congruent condition. Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fl_rt_inc_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flanker task. Log-transformed Average response time on correct trials of the incongruent condition. Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">si_score_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simon task. Log-transformed Congruency effect based on mean response times of correct trials (congruent - incongruent). Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">si_rt_con_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simon task. Log-transformed Average response time on correct trials of the congruent condition. Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">si_rt_inc_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simon task. Log-transformed Average response time on correct trials of the incongruent condition. Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cs_score_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color-shape task. Log-transformed Switch cost based on mean response times of correct trials, excluding trials following an error (repeat - switch). Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cs_rt_rep_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color-shape task. Log-transformed Average response time on correct trials of the repeat condition. Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cs_rt_sw_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color-shape task. Log-transformed Average response time on correct trials of the switch condition. Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gl_score_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global-Localtask. Log-transformed Switch cost based on mean response times of correct trials, excluding trials following an error (repeat - switch). Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gl_rt_rep_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global-Local task. Log-transformed Average response time on correct trials of the repeat condition. Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gl_rt_sw_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global-Localtask. Log-transformed Average response time on correct trials of the switch condition. Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as_score_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Animacy-Size task. Log-transformed Switch cost based on mean response times of correct trials, excluding trials following an error (repeat - switch). Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as_rt_rep_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Animacy-Size task. Log-transformed Average response time on correct trials of the repeat condition. Corrected for noise and state anxiety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as_rt_sw_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Animacy-Size task. Log-transformed Average response time on correct trials of the switch condition. Corrected for noise and state anxiety</t>
+  </si>
+  <si>
     <t xml:space="preserve">fl_a1</t>
   </si>
   <si>
@@ -363,6 +483,186 @@
   </si>
   <si>
     <t xml:space="preserve">Animacy-Size task. Non-decision time of switch condition (derived from the Drift Diffusion Model)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fl_v1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flanker task. Drift rate of congruent condition (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fl_v2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flanker task. Drift rate of incongruent condition  (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fl_a1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flanker task. Boundary separation of congruent condition (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fl_a2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flanker task. Boundary separation of incongruent condition (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fl_t1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flanker task. Non-decision time of congruent condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">fl_t2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flanker task. Non-decision time of incongruent condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">si_v1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simon task. Drift rate of congruent condition  (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">si_v2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simon task. Drift rate of incongruent condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">si_a1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simon task. Boundary separation of congruent condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">si_a2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simon task. Boundary separation of incongruent condition  (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">si_t1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simon task. Non-decision time of congruent condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">si_t2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simon task. Non-decision time of incongruent condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cs_v1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color-shape task. Drift rate of repeat condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cs_v2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color-shape task. Drift rate of switch condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cs_a1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color-shape task. Boundary separation of repeat condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cs_a2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color-shape task. Boundary separation of switch condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cs_t1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color-shape task. Non-decision time of repeat condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cs_t2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color-shape task. Non-decision time of switch condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">gl_v1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global-Local task. Drift rate of repeat condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">gl_v2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global-Local task. Drift rate of switch condition (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gl_a1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global-Local task. Boundary separation of repeat condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">gl_a2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global-Local task. Boundary separation of switch condition (corrected for noise and state anxiety) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">gl_t1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global-Local task. Non-decision time of repeat condition (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gl_t2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global-Local task. Non-decision time of switch condition (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as_v1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Animacy-Size task. Drift rate of repeat condition (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as_v2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Animacy-Size task. Drift rate of switch condition (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as_a1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Animacy-Size task. Boundary separation of repeat condition (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as_a2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Animacy-Size task. Boundary separation of switch condition (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as_t1_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Animacy-Size task. Non-decision time of repeat condition (corrected for noise and state anxiety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as_t2_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Animacy-Size task. Non-decision time of switch condition (corrected for noise and state anxiety)</t>
   </si>
 </sst>
 </file>
@@ -691,8 +991,8 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="12.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="132.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="21.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="187.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="250.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
@@ -998,7 +1298,7 @@
         <v>57</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>5</v>
       </c>
       <c r="C28" t="s">
         <v>5</v>
@@ -1006,10 +1306,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B29" t="s">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="C29" t="s">
         <v>5</v>
@@ -1017,10 +1317,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="C30" t="s">
         <v>5</v>
@@ -1028,10 +1328,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B31" t="s">
-        <v>64</v>
+        <v>5</v>
       </c>
       <c r="C31" t="s">
         <v>5</v>
@@ -1039,10 +1339,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="C32" t="s">
         <v>5</v>
@@ -1050,10 +1350,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B33" t="s">
-        <v>68</v>
+        <v>5</v>
       </c>
       <c r="C33" t="s">
         <v>5</v>
@@ -1061,10 +1361,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B34" t="s">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="C34" t="s">
         <v>5</v>
@@ -1072,10 +1372,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="B35" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="C35" t="s">
         <v>5</v>
@@ -1083,10 +1383,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B36" t="s">
-        <v>74</v>
+        <v>5</v>
       </c>
       <c r="C36" t="s">
         <v>5</v>
@@ -1094,10 +1394,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>5</v>
       </c>
       <c r="C37" t="s">
         <v>5</v>
@@ -1105,10 +1405,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="B38" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="C38" t="s">
         <v>5</v>
@@ -1116,10 +1416,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="B39" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C39" t="s">
         <v>5</v>
@@ -1127,10 +1427,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B40" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="C40" t="s">
         <v>5</v>
@@ -1138,10 +1438,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="B41" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="C41" t="s">
         <v>5</v>
@@ -1149,10 +1449,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B42" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="C42" t="s">
         <v>5</v>
@@ -1160,10 +1460,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B43" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="C43" t="s">
         <v>5</v>
@@ -1171,10 +1471,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="B44" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="C44" t="s">
         <v>5</v>
@@ -1182,10 +1482,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="B45" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="C45" t="s">
         <v>5</v>
@@ -1193,10 +1493,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B46" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C46" t="s">
         <v>5</v>
@@ -1204,10 +1504,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B47" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="C47" t="s">
         <v>5</v>
@@ -1215,10 +1515,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B48" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C48" t="s">
         <v>5</v>
@@ -1226,10 +1526,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="B49" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C49" t="s">
         <v>5</v>
@@ -1237,10 +1537,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="B50" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="C50" t="s">
         <v>5</v>
@@ -1248,10 +1548,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B51" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C51" t="s">
         <v>5</v>
@@ -1259,10 +1559,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="B52" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="C52" t="s">
         <v>5</v>
@@ -1270,10 +1570,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B53" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C53" t="s">
         <v>5</v>
@@ -1281,10 +1581,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="B54" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C54" t="s">
         <v>5</v>
@@ -1292,10 +1592,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B55" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C55" t="s">
         <v>5</v>
@@ -1303,10 +1603,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="B56" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C56" t="s">
         <v>5</v>
@@ -1314,12 +1614,617 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
+        <v>105</v>
+      </c>
+      <c r="B57" t="s">
+        <v>106</v>
+      </c>
+      <c r="C57" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>107</v>
+      </c>
+      <c r="B58" t="s">
+        <v>108</v>
+      </c>
+      <c r="C58" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>109</v>
+      </c>
+      <c r="B59" t="s">
+        <v>110</v>
+      </c>
+      <c r="C59" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>111</v>
+      </c>
+      <c r="B60" t="s">
+        <v>112</v>
+      </c>
+      <c r="C60" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>113</v>
+      </c>
+      <c r="B61" t="s">
+        <v>114</v>
+      </c>
+      <c r="C61" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
         <v>115</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B62" t="s">
         <v>116</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C62" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>117</v>
+      </c>
+      <c r="B63" t="s">
+        <v>118</v>
+      </c>
+      <c r="C63" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>119</v>
+      </c>
+      <c r="B64" t="s">
+        <v>120</v>
+      </c>
+      <c r="C64" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>121</v>
+      </c>
+      <c r="B65" t="s">
+        <v>122</v>
+      </c>
+      <c r="C65" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>123</v>
+      </c>
+      <c r="B66" t="s">
+        <v>124</v>
+      </c>
+      <c r="C66" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>125</v>
+      </c>
+      <c r="B67" t="s">
+        <v>126</v>
+      </c>
+      <c r="C67" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>127</v>
+      </c>
+      <c r="B68" t="s">
+        <v>128</v>
+      </c>
+      <c r="C68" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>129</v>
+      </c>
+      <c r="B69" t="s">
+        <v>130</v>
+      </c>
+      <c r="C69" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>131</v>
+      </c>
+      <c r="B70" t="s">
+        <v>132</v>
+      </c>
+      <c r="C70" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>133</v>
+      </c>
+      <c r="B71" t="s">
+        <v>134</v>
+      </c>
+      <c r="C71" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>135</v>
+      </c>
+      <c r="B72" t="s">
+        <v>136</v>
+      </c>
+      <c r="C72" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>137</v>
+      </c>
+      <c r="B73" t="s">
+        <v>138</v>
+      </c>
+      <c r="C73" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s">
+        <v>139</v>
+      </c>
+      <c r="B74" t="s">
+        <v>140</v>
+      </c>
+      <c r="C74" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s">
+        <v>141</v>
+      </c>
+      <c r="B75" t="s">
+        <v>142</v>
+      </c>
+      <c r="C75" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s">
+        <v>143</v>
+      </c>
+      <c r="B76" t="s">
+        <v>144</v>
+      </c>
+      <c r="C76" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s">
+        <v>145</v>
+      </c>
+      <c r="B77" t="s">
+        <v>146</v>
+      </c>
+      <c r="C77" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s">
+        <v>147</v>
+      </c>
+      <c r="B78" t="s">
+        <v>148</v>
+      </c>
+      <c r="C78" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s">
+        <v>149</v>
+      </c>
+      <c r="B79" t="s">
+        <v>150</v>
+      </c>
+      <c r="C79" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
+        <v>151</v>
+      </c>
+      <c r="B80" t="s">
+        <v>152</v>
+      </c>
+      <c r="C80" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s">
+        <v>153</v>
+      </c>
+      <c r="B81" t="s">
+        <v>154</v>
+      </c>
+      <c r="C81" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s">
+        <v>155</v>
+      </c>
+      <c r="B82" t="s">
+        <v>156</v>
+      </c>
+      <c r="C82" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s">
+        <v>157</v>
+      </c>
+      <c r="B83" t="s">
+        <v>158</v>
+      </c>
+      <c r="C83" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s">
+        <v>159</v>
+      </c>
+      <c r="B84" t="s">
+        <v>160</v>
+      </c>
+      <c r="C84" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s">
+        <v>161</v>
+      </c>
+      <c r="B85" t="s">
+        <v>162</v>
+      </c>
+      <c r="C85" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s">
+        <v>163</v>
+      </c>
+      <c r="B86" t="s">
+        <v>164</v>
+      </c>
+      <c r="C86" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="s">
+        <v>165</v>
+      </c>
+      <c r="B87" t="s">
+        <v>166</v>
+      </c>
+      <c r="C87" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="s">
+        <v>167</v>
+      </c>
+      <c r="B88" t="s">
+        <v>168</v>
+      </c>
+      <c r="C88" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="s">
+        <v>169</v>
+      </c>
+      <c r="B89" t="s">
+        <v>170</v>
+      </c>
+      <c r="C89" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="s">
+        <v>171</v>
+      </c>
+      <c r="B90" t="s">
+        <v>172</v>
+      </c>
+      <c r="C90" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="s">
+        <v>173</v>
+      </c>
+      <c r="B91" t="s">
+        <v>174</v>
+      </c>
+      <c r="C91" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="s">
+        <v>175</v>
+      </c>
+      <c r="B92" t="s">
+        <v>176</v>
+      </c>
+      <c r="C92" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="s">
+        <v>177</v>
+      </c>
+      <c r="B93" t="s">
+        <v>178</v>
+      </c>
+      <c r="C93" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="s">
+        <v>179</v>
+      </c>
+      <c r="B94" t="s">
+        <v>180</v>
+      </c>
+      <c r="C94" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="s">
+        <v>181</v>
+      </c>
+      <c r="B95" t="s">
+        <v>182</v>
+      </c>
+      <c r="C95" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="s">
+        <v>183</v>
+      </c>
+      <c r="B96" t="s">
+        <v>184</v>
+      </c>
+      <c r="C96" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="s">
+        <v>185</v>
+      </c>
+      <c r="B97" t="s">
+        <v>186</v>
+      </c>
+      <c r="C97" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="s">
+        <v>187</v>
+      </c>
+      <c r="B98" t="s">
+        <v>188</v>
+      </c>
+      <c r="C98" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="s">
+        <v>189</v>
+      </c>
+      <c r="B99" t="s">
+        <v>190</v>
+      </c>
+      <c r="C99" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="s">
+        <v>191</v>
+      </c>
+      <c r="B100" t="s">
+        <v>192</v>
+      </c>
+      <c r="C100" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="s">
+        <v>193</v>
+      </c>
+      <c r="B101" t="s">
+        <v>194</v>
+      </c>
+      <c r="C101" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="s">
+        <v>195</v>
+      </c>
+      <c r="B102" t="s">
+        <v>196</v>
+      </c>
+      <c r="C102" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="s">
+        <v>197</v>
+      </c>
+      <c r="B103" t="s">
+        <v>198</v>
+      </c>
+      <c r="C103" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="s">
+        <v>199</v>
+      </c>
+      <c r="B104" t="s">
+        <v>200</v>
+      </c>
+      <c r="C104" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="s">
+        <v>201</v>
+      </c>
+      <c r="B105" t="s">
+        <v>202</v>
+      </c>
+      <c r="C105" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s">
+        <v>203</v>
+      </c>
+      <c r="B106" t="s">
+        <v>204</v>
+      </c>
+      <c r="C106" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="s">
+        <v>205</v>
+      </c>
+      <c r="B107" t="s">
+        <v>206</v>
+      </c>
+      <c r="C107" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s">
+        <v>207</v>
+      </c>
+      <c r="B108" t="s">
+        <v>208</v>
+      </c>
+      <c r="C108" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="s">
+        <v>209</v>
+      </c>
+      <c r="B109" t="s">
+        <v>210</v>
+      </c>
+      <c r="C109" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s">
+        <v>211</v>
+      </c>
+      <c r="B110" t="s">
+        <v>212</v>
+      </c>
+      <c r="C110" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s">
+        <v>213</v>
+      </c>
+      <c r="B111" t="s">
+        <v>214</v>
+      </c>
+      <c r="C111" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s">
+        <v>215</v>
+      </c>
+      <c r="B112" t="s">
+        <v>216</v>
+      </c>
+      <c r="C112" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Final commit prior to first submission
</commit_message>
<xml_diff>
--- a/1_data/3_AnalysisData/MetaData/codebook_AnalysisData.xlsx
+++ b/1_data/3_AnalysisData/MetaData/codebook_AnalysisData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="218">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -86,13 +86,16 @@
     <t xml:space="preserve">urb</t>
   </si>
   <si>
+    <t xml:space="preserve">Urban character of place of residence (based on surrounding address density per km^2^</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extremely urban (2,500 or more) = 1, Very urban (1,500 to 2,500) = 2, Moderately urban (1,000 to 1,500) = 3, Slightly urban (500 to 1,000) = 4, Not urban (less than 500) = 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">urb_c</t>
+  </si>
+  <si>
     <t xml:space="preserve">Urban character of place of residence; centered</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extremely urban (2,500 or more) = 1, Very urban (1,500 to 2,500) = 2, Moderately urban (1,000 to 1,500) = 3, Slightly urban (500 to 1,000) = 4, Not urban (less than 500) = 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">urb_c</t>
   </si>
   <si>
     <t xml:space="preserve">fl_score</t>
@@ -1122,7 +1125,7 @@
         <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
         <v>5</v>
@@ -1130,10 +1133,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
         <v>5</v>
@@ -1141,10 +1144,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
         <v>5</v>
@@ -1152,10 +1155,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C15" t="s">
         <v>5</v>
@@ -1163,10 +1166,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C16" t="s">
         <v>5</v>
@@ -1174,10 +1177,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C17" t="s">
         <v>5</v>
@@ -1185,10 +1188,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
         <v>5</v>
@@ -1196,10 +1199,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
         <v>5</v>
@@ -1207,10 +1210,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
         <v>5</v>
@@ -1218,10 +1221,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C21" t="s">
         <v>5</v>
@@ -1229,10 +1232,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C22" t="s">
         <v>5</v>
@@ -1240,10 +1243,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C23" t="s">
         <v>5</v>
@@ -1251,10 +1254,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B24" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C24" t="s">
         <v>5</v>
@@ -1262,10 +1265,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C25" t="s">
         <v>5</v>
@@ -1273,10 +1276,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B26" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C26" t="s">
         <v>5</v>
@@ -1284,10 +1287,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C27" t="s">
         <v>5</v>
@@ -1295,7 +1298,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B28" t="s">
         <v>5</v>
@@ -1306,7 +1309,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B29" t="s">
         <v>5</v>
@@ -1317,7 +1320,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B30" t="s">
         <v>5</v>
@@ -1328,7 +1331,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B31" t="s">
         <v>5</v>
@@ -1339,7 +1342,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B32" t="s">
         <v>5</v>
@@ -1350,7 +1353,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B33" t="s">
         <v>5</v>
@@ -1361,7 +1364,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B34" t="s">
         <v>5</v>
@@ -1372,7 +1375,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B35" t="s">
         <v>5</v>
@@ -1383,7 +1386,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B36" t="s">
         <v>5</v>
@@ -1394,7 +1397,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B37" t="s">
         <v>5</v>
@@ -1405,10 +1408,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B38" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C38" t="s">
         <v>5</v>
@@ -1416,10 +1419,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B39" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C39" t="s">
         <v>5</v>
@@ -1427,10 +1430,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B40" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C40" t="s">
         <v>5</v>
@@ -1438,10 +1441,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B41" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C41" t="s">
         <v>5</v>
@@ -1449,10 +1452,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B42" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C42" t="s">
         <v>5</v>
@@ -1460,10 +1463,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B43" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C43" t="s">
         <v>5</v>
@@ -1471,10 +1474,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B44" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C44" t="s">
         <v>5</v>
@@ -1482,10 +1485,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B45" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C45" t="s">
         <v>5</v>
@@ -1493,10 +1496,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B46" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C46" t="s">
         <v>5</v>
@@ -1504,10 +1507,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B47" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C47" t="s">
         <v>5</v>
@@ -1515,10 +1518,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B48" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C48" t="s">
         <v>5</v>
@@ -1526,10 +1529,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B49" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C49" t="s">
         <v>5</v>
@@ -1537,10 +1540,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B50" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C50" t="s">
         <v>5</v>
@@ -1548,10 +1551,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B51" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C51" t="s">
         <v>5</v>
@@ -1559,10 +1562,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B52" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C52" t="s">
         <v>5</v>
@@ -1570,10 +1573,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B53" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C53" t="s">
         <v>5</v>
@@ -1581,10 +1584,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B54" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C54" t="s">
         <v>5</v>
@@ -1592,10 +1595,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B55" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C55" t="s">
         <v>5</v>
@@ -1603,10 +1606,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B56" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C56" t="s">
         <v>5</v>
@@ -1614,10 +1617,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B57" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C57" t="s">
         <v>5</v>
@@ -1625,10 +1628,10 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B58" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C58" t="s">
         <v>5</v>
@@ -1636,10 +1639,10 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B59" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C59" t="s">
         <v>5</v>
@@ -1647,10 +1650,10 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B60" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C60" t="s">
         <v>5</v>
@@ -1658,10 +1661,10 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B61" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C61" t="s">
         <v>5</v>
@@ -1669,10 +1672,10 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B62" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C62" t="s">
         <v>5</v>
@@ -1680,10 +1683,10 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B63" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C63" t="s">
         <v>5</v>
@@ -1691,10 +1694,10 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B64" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C64" t="s">
         <v>5</v>
@@ -1702,10 +1705,10 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B65" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C65" t="s">
         <v>5</v>
@@ -1713,10 +1716,10 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B66" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C66" t="s">
         <v>5</v>
@@ -1724,10 +1727,10 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B67" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C67" t="s">
         <v>5</v>
@@ -1735,10 +1738,10 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B68" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C68" t="s">
         <v>5</v>
@@ -1746,10 +1749,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B69" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C69" t="s">
         <v>5</v>
@@ -1757,10 +1760,10 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B70" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C70" t="s">
         <v>5</v>
@@ -1768,10 +1771,10 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B71" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C71" t="s">
         <v>5</v>
@@ -1779,10 +1782,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B72" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C72" t="s">
         <v>5</v>
@@ -1790,10 +1793,10 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B73" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C73" t="s">
         <v>5</v>
@@ -1801,10 +1804,10 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B74" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C74" t="s">
         <v>5</v>
@@ -1812,10 +1815,10 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B75" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C75" t="s">
         <v>5</v>
@@ -1823,10 +1826,10 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B76" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C76" t="s">
         <v>5</v>
@@ -1834,10 +1837,10 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B77" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C77" t="s">
         <v>5</v>
@@ -1845,10 +1848,10 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B78" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C78" t="s">
         <v>5</v>
@@ -1856,10 +1859,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B79" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C79" t="s">
         <v>5</v>
@@ -1867,10 +1870,10 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B80" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C80" t="s">
         <v>5</v>
@@ -1878,10 +1881,10 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B81" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C81" t="s">
         <v>5</v>
@@ -1889,10 +1892,10 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B82" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C82" t="s">
         <v>5</v>
@@ -1900,10 +1903,10 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B83" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C83" t="s">
         <v>5</v>
@@ -1911,10 +1914,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B84" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C84" t="s">
         <v>5</v>
@@ -1922,10 +1925,10 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B85" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C85" t="s">
         <v>5</v>
@@ -1933,10 +1936,10 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B86" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C86" t="s">
         <v>5</v>
@@ -1944,10 +1947,10 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B87" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C87" t="s">
         <v>5</v>
@@ -1955,10 +1958,10 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B88" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C88" t="s">
         <v>5</v>
@@ -1966,10 +1969,10 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B89" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C89" t="s">
         <v>5</v>
@@ -1977,10 +1980,10 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B90" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C90" t="s">
         <v>5</v>
@@ -1988,10 +1991,10 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B91" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C91" t="s">
         <v>5</v>
@@ -1999,10 +2002,10 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B92" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C92" t="s">
         <v>5</v>
@@ -2010,10 +2013,10 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B93" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C93" t="s">
         <v>5</v>
@@ -2021,10 +2024,10 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B94" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C94" t="s">
         <v>5</v>
@@ -2032,10 +2035,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B95" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C95" t="s">
         <v>5</v>
@@ -2043,10 +2046,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B96" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C96" t="s">
         <v>5</v>
@@ -2054,10 +2057,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B97" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C97" t="s">
         <v>5</v>
@@ -2065,10 +2068,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B98" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C98" t="s">
         <v>5</v>
@@ -2076,10 +2079,10 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B99" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C99" t="s">
         <v>5</v>
@@ -2087,10 +2090,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B100" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C100" t="s">
         <v>5</v>
@@ -2098,10 +2101,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B101" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C101" t="s">
         <v>5</v>
@@ -2109,10 +2112,10 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B102" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C102" t="s">
         <v>5</v>
@@ -2120,10 +2123,10 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B103" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C103" t="s">
         <v>5</v>
@@ -2131,10 +2134,10 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B104" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C104" t="s">
         <v>5</v>
@@ -2142,10 +2145,10 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B105" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C105" t="s">
         <v>5</v>
@@ -2153,10 +2156,10 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B106" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C106" t="s">
         <v>5</v>
@@ -2164,10 +2167,10 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B107" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C107" t="s">
         <v>5</v>
@@ -2175,10 +2178,10 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B108" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C108" t="s">
         <v>5</v>
@@ -2186,10 +2189,10 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B109" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C109" t="s">
         <v>5</v>
@@ -2197,10 +2200,10 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B110" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C110" t="s">
         <v>5</v>
@@ -2208,10 +2211,10 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B111" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C111" t="s">
         <v>5</v>
@@ -2219,10 +2222,10 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B112" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C112" t="s">
         <v>5</v>

</xml_diff>